<commit_message>
Ordenamiento de plantilla y librerias utilizadas, Creacion de tabla Cliente, Cambio de valores para conexion a base de datos, Se estabiliza funcionalidad de consultar clientes
</commit_message>
<xml_diff>
--- a/DB/CHOLITOS_GYM_SCRIPT_MASIVOS.xlsx
+++ b/DB/CHOLITOS_GYM_SCRIPT_MASIVOS.xlsx
@@ -24,10 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="51">
-  <si>
-    <t>CODIGO_GENERACION</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>PRIMER_NOMBRE</t>
   </si>
@@ -44,12 +41,6 @@
     <t>APELLIDO_CASADA</t>
   </si>
   <si>
-    <t>FECHA_PAGO</t>
-  </si>
-  <si>
-    <t>FIRMA</t>
-  </si>
-  <si>
     <t>SPK5C</t>
   </si>
   <si>
@@ -71,9 +62,6 @@
     <t>Silva</t>
   </si>
   <si>
-    <t>S</t>
-  </si>
-  <si>
     <t>Alexis</t>
   </si>
   <si>
@@ -107,9 +95,6 @@
     <t>Genovez</t>
   </si>
   <si>
-    <t>N</t>
-  </si>
-  <si>
     <t>RXZ1E</t>
   </si>
   <si>
@@ -122,61 +107,10 @@
     <t>Sambrano</t>
   </si>
   <si>
-    <t>2024$12$02</t>
-  </si>
-  <si>
-    <t>2024$12$03</t>
-  </si>
-  <si>
-    <t>2024$12$04</t>
-  </si>
-  <si>
-    <t>2024$12$05</t>
-  </si>
-  <si>
-    <t>2024$12$06</t>
-  </si>
-  <si>
-    <t>2024$12$07</t>
-  </si>
-  <si>
-    <t>2024$12$08</t>
-  </si>
-  <si>
-    <t>2024$12$09</t>
-  </si>
-  <si>
-    <t>2024$12$10</t>
-  </si>
-  <si>
-    <t>2024$12$11</t>
-  </si>
-  <si>
-    <t>2024$12$31</t>
-  </si>
-  <si>
-    <t>2025$01$07</t>
-  </si>
-  <si>
-    <t>2025$01$08</t>
-  </si>
-  <si>
-    <t>2025$01$09</t>
-  </si>
-  <si>
-    <t>FECHA_INICIO</t>
-  </si>
-  <si>
-    <t>FECHA_FIN</t>
-  </si>
-  <si>
-    <t>TIPO_MODALIDAD</t>
-  </si>
-  <si>
-    <t>M</t>
-  </si>
-  <si>
     <t>INSERT PARA CLIENTES</t>
+  </si>
+  <si>
+    <t>CODIGO_GIMNASIO</t>
   </si>
 </sst>
 </file>
@@ -220,9 +154,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -244,20 +177,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:K8" totalsRowShown="0">
-  <autoFilter ref="A1:K8"/>
-  <tableColumns count="11">
-    <tableColumn id="1" name="CODIGO_GENERACION"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:F8" totalsRowShown="0">
+  <autoFilter ref="A1:F8"/>
+  <tableColumns count="6">
+    <tableColumn id="1" name="CODIGO_GIMNASIO"/>
     <tableColumn id="2" name="PRIMER_NOMBRE"/>
     <tableColumn id="3" name="SEGUNDO_NOMBRE"/>
     <tableColumn id="4" name="PRIMER_APELLIDO"/>
     <tableColumn id="5" name="SEGUNDO_APELLIDO"/>
     <tableColumn id="6" name="APELLIDO_CASADA"/>
-    <tableColumn id="7" name="FECHA_PAGO"/>
-    <tableColumn id="8" name="FECHA_INICIO"/>
-    <tableColumn id="9" name="FECHA_FIN"/>
-    <tableColumn id="10" name="FIRMA"/>
-    <tableColumn id="12" name="TIPO_MODALIDAD"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -526,7 +454,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.33203125" bestFit="1" customWidth="1"/>
@@ -545,249 +473,135 @@
     <col min="14" max="14" width="11.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" t="str">
+        <f>"INSERT INTO Cliente(CodigoGimnasio, PrimerNombre, SegundoNombre, PrimerApellido, SegundoApellido, ApellidoCasada) VALUES('"&amp;A2&amp;"', '"&amp;B2&amp;"', '"&amp;C2&amp;"', '"&amp;D2&amp;"', '"&amp;E2&amp;"', '"&amp;F2&amp;"');"</f>
+        <v>INSERT INTO Cliente(CodigoGimnasio, PrimerNombre, SegundoNombre, PrimerApellido, SegundoApellido, ApellidoCasada) VALUES('SPK5C', 'Damaris', '', 'Silva', '', '');</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
-        <v>46</v>
-      </c>
-      <c r="I1" t="s">
-        <v>47</v>
-      </c>
-      <c r="J1" t="s">
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" t="str">
+        <f t="shared" ref="H3:H8" si="0">"INSERT INTO Cliente(CodigoGimnasio, PrimerNombre, SegundoNombre, PrimerApellido, SegundoApellido, ApellidoCasada) VALUES('"&amp;A3&amp;"', '"&amp;B3&amp;"', '"&amp;C3&amp;"', '"&amp;D3&amp;"', '"&amp;E3&amp;"', '"&amp;F3&amp;"');"</f>
+        <v>INSERT INTO Cliente(CodigoGimnasio, PrimerNombre, SegundoNombre, PrimerApellido, SegundoApellido, ApellidoCasada) VALUES('L1CWT', 'Alexis', '', 'Castaneda', '', '');</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>7</v>
       </c>
-      <c r="K1" t="s">
-        <v>48</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" t="str">
+        <f t="shared" si="0"/>
+        <v>INSERT INTO Cliente(CodigoGimnasio, PrimerNombre, SegundoNombre, PrimerApellido, SegundoApellido, ApellidoCasada) VALUES('KEAPS', 'Sara', '', '', '', 'de Clemente');</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="J2" t="s">
-        <v>15</v>
-      </c>
-      <c r="K2" t="s">
-        <v>49</v>
-      </c>
-      <c r="M2" t="str">
-        <f>"INSERT INTO CHOLITOS_GYM_CLIENTE(CODIGO_GENERACION, PRIMER_NOMBRE, SEGUNDO_NOMBRE, PRIMER_APELLIDO, SEGUNDO_APELLIDO, APELLIDO_CASADA, FECHA_PAGO, FECHA_INICIO, FECHA_FIN, FIRMA, TIPO_MODALIDAD) VALUES('"&amp;A2&amp;"', '"&amp;B2&amp;"', '"&amp;C2&amp;"', '"&amp;D2&amp;"', '"&amp;E2&amp;"', '"&amp;F2&amp;"', '"&amp;G2&amp;"', '"&amp;H2&amp;"', '"&amp;I2&amp;"', '"&amp;J2&amp;"', '"&amp;K2&amp;"');"</f>
-        <v>INSERT INTO CHOLITOS_GYM_CLIENTE(CODIGO_GENERACION, PRIMER_NOMBRE, SEGUNDO_NOMBRE, PRIMER_APELLIDO, SEGUNDO_APELLIDO, APELLIDO_CASADA, FECHA_PAGO, FECHA_INICIO, FECHA_FIN, FIRMA, TIPO_MODALIDAD) VALUES('SPK5C', 'Damaris', '', 'Silva', '', '', '2024$12$02', '2024$12$02', '2024$12$31', 'S', 'M');</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" t="str">
+        <f t="shared" si="0"/>
+        <v>INSERT INTO Cliente(CodigoGimnasio, PrimerNombre, SegundoNombre, PrimerApellido, SegundoApellido, ApellidoCasada) VALUES('KTGQ9', 'Stanley', '', 'Idalgo', '', '');</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>9</v>
       </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="J3" t="s">
-        <v>15</v>
-      </c>
-      <c r="K3" t="s">
-        <v>49</v>
-      </c>
-      <c r="M3" t="str">
-        <f t="shared" ref="M3:M8" si="0">"INSERT INTO CHOLITOS_GYM_CLIENTE(CODIGO_GENERACION, PRIMER_NOMBRE, SEGUNDO_NOMBRE, PRIMER_APELLIDO, SEGUNDO_APELLIDO, APELLIDO_CASADA, FECHA_PAGO, FECHA_INICIO, FECHA_FIN, FIRMA, TIPO_MODALIDAD) VALUES('"&amp;A3&amp;"', '"&amp;B3&amp;"', '"&amp;C3&amp;"', '"&amp;D3&amp;"', '"&amp;E3&amp;"', '"&amp;F3&amp;"', '"&amp;G3&amp;"', '"&amp;H3&amp;"', '"&amp;I3&amp;"', '"&amp;J3&amp;"', '"&amp;K3&amp;"');"</f>
-        <v>INSERT INTO CHOLITOS_GYM_CLIENTE(CODIGO_GENERACION, PRIMER_NOMBRE, SEGUNDO_NOMBRE, PRIMER_APELLIDO, SEGUNDO_APELLIDO, APELLIDO_CASADA, FECHA_PAGO, FECHA_INICIO, FECHA_FIN, FIRMA, TIPO_MODALIDAD) VALUES('L1CWT', 'Alexis', '', 'Castaneda', '', '', '2024$12$03', '2024$12$03', '2024$12$31', 'S', 'M');</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="B6" t="s">
         <v>18</v>
       </c>
-      <c r="F4" t="s">
+      <c r="D6" t="s">
         <v>19</v>
       </c>
-      <c r="G4" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="J4" t="s">
-        <v>15</v>
-      </c>
-      <c r="K4" t="s">
-        <v>49</v>
-      </c>
-      <c r="M4" t="str">
+      <c r="E6" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO CHOLITOS_GYM_CLIENTE(CODIGO_GENERACION, PRIMER_NOMBRE, SEGUNDO_NOMBRE, PRIMER_APELLIDO, SEGUNDO_APELLIDO, APELLIDO_CASADA, FECHA_PAGO, FECHA_INICIO, FECHA_FIN, FIRMA, TIPO_MODALIDAD) VALUES('KEAPS', 'Sara', '', '', '', 'de Clemente', '2024$12$04', '2024$12$04', '2024$12$31', 'S', 'M');</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" t="s">
+        <v>INSERT INTO Cliente(CodigoGimnasio, PrimerNombre, SegundoNombre, PrimerApellido, SegundoApellido, ApellidoCasada) VALUES('RHD1E', 'Israel ', '', 'Cabrera', 'Rodriguez', '');</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" t="s">
         <v>21</v>
       </c>
-      <c r="G5" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="J5" t="s">
-        <v>15</v>
-      </c>
-      <c r="K5" t="s">
-        <v>49</v>
-      </c>
-      <c r="M5" t="str">
+      <c r="D7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO CHOLITOS_GYM_CLIENTE(CODIGO_GENERACION, PRIMER_NOMBRE, SEGUNDO_NOMBRE, PRIMER_APELLIDO, SEGUNDO_APELLIDO, APELLIDO_CASADA, FECHA_PAGO, FECHA_INICIO, FECHA_FIN, FIRMA, TIPO_MODALIDAD) VALUES('KTGQ9', 'Stanley', '', 'Idalgo', '', '', '2024$12$05', '', '', 'S', 'M');</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" t="s">
-        <v>23</v>
-      </c>
-      <c r="E6" t="s">
+        <v>INSERT INTO Cliente(CodigoGimnasio, PrimerNombre, SegundoNombre, PrimerApellido, SegundoApellido, ApellidoCasada) VALUES('RXZ1E', 'Nestor', '', 'Genovez', '', '');</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="J6" t="s">
-        <v>15</v>
-      </c>
-      <c r="K6" t="s">
-        <v>49</v>
-      </c>
-      <c r="M6" t="str">
+      <c r="B8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" t="s">
+        <v>26</v>
+      </c>
+      <c r="H8" t="str">
         <f t="shared" si="0"/>
-        <v>INSERT INTO CHOLITOS_GYM_CLIENTE(CODIGO_GENERACION, PRIMER_NOMBRE, SEGUNDO_NOMBRE, PRIMER_APELLIDO, SEGUNDO_APELLIDO, APELLIDO_CASADA, FECHA_PAGO, FECHA_INICIO, FECHA_FIN, FIRMA, TIPO_MODALIDAD) VALUES('RHD1E', 'Israel ', '', 'Cabrera', 'Rodriguez', '', '2024$12$06', '2024$12$09', '2025$01$07', 'S', 'M');</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="J7" t="s">
-        <v>27</v>
-      </c>
-      <c r="K7" t="s">
-        <v>49</v>
-      </c>
-      <c r="M7" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO CHOLITOS_GYM_CLIENTE(CODIGO_GENERACION, PRIMER_NOMBRE, SEGUNDO_NOMBRE, PRIMER_APELLIDO, SEGUNDO_APELLIDO, APELLIDO_CASADA, FECHA_PAGO, FECHA_INICIO, FECHA_FIN, FIRMA, TIPO_MODALIDAD) VALUES('RXZ1E', 'Nestor', '', 'Genovez', '', '', '2024$12$07', '2024$12$10', '2025$01$08', 'N', 'M');</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" t="s">
-        <v>30</v>
-      </c>
-      <c r="D8" t="s">
-        <v>31</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="J8" t="s">
-        <v>27</v>
-      </c>
-      <c r="K8" t="s">
-        <v>49</v>
-      </c>
-      <c r="M8" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO CHOLITOS_GYM_CLIENTE(CODIGO_GENERACION, PRIMER_NOMBRE, SEGUNDO_NOMBRE, PRIMER_APELLIDO, SEGUNDO_APELLIDO, APELLIDO_CASADA, FECHA_PAGO, FECHA_INICIO, FECHA_FIN, FIRMA, TIPO_MODALIDAD) VALUES('R2L1E', 'Mabel', '', 'Sambrano', '', '', '2024$12$08', '2024$12$11', '2025$01$09', 'N', 'M');</v>
+        <v>INSERT INTO Cliente(CodigoGimnasio, PrimerNombre, SegundoNombre, PrimerApellido, SegundoApellido, ApellidoCasada) VALUES('R2L1E', 'Mabel', '', 'Sambrano', '', '');</v>
       </c>
     </row>
   </sheetData>

</xml_diff>